<commit_message>
Tracker: replace MAXIFS with SUMPRODUCT/MAX for Google Sheets compatibility
The latest-value block used _xlfn.MAXIFS, which Google Sheets does not
reliably resolve on import. SUMPRODUCT(MAX(...)) evaluates natively in
Excel, LibreOffice and Google Sheets without an array entry or a prefix.
LibreOffice headless recalculation timed out in this environment at 60s,
300s and 579s, so the formulas were verified by computing their expected
results in Python instead: 28 tasks, P0/P1/P2 = 8/11/9, and all 30 metrics
in the tracking log resolvable by the latest-value block.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MUHUj2RPRZAnBNADpTZfsW
</commit_message>
<xml_diff>
--- a/docs/seo/designbees-aeo-seo-tracker-2026-09-10.xlsx
+++ b/docs/seo/designbees-aeo-seo-tracker-2026-09-10.xlsx
@@ -3709,7 +3709,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:L199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3814,11 +3814,11 @@
         </is>
       </c>
       <c r="H5" s="7">
-        <f>SUMIFS($D$5:$D$1000,$C$5:$C$1000,G5,$A$5:$A$1000,_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G5))</f>
+        <f>IF(I5=0,"",SUMIFS($D$5:$D$1000,$C$5:$C$1000,G5,$A$5:$A$1000,I5))</f>
         <v/>
       </c>
       <c r="I5" s="11">
-        <f>_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G5)</f>
+        <f>SUMPRODUCT(MAX(($C$5:$C$1000=G5)*$A$5:$A$1000))</f>
         <v/>
       </c>
     </row>
@@ -3846,11 +3846,11 @@
         </is>
       </c>
       <c r="H6" s="7">
-        <f>SUMIFS($D$5:$D$1000,$C$5:$C$1000,G6,$A$5:$A$1000,_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G6))</f>
+        <f>IF(I6=0,"",SUMIFS($D$5:$D$1000,$C$5:$C$1000,G6,$A$5:$A$1000,I6))</f>
         <v/>
       </c>
       <c r="I6" s="11">
-        <f>_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G6)</f>
+        <f>SUMPRODUCT(MAX(($C$5:$C$1000=G6)*$A$5:$A$1000))</f>
         <v/>
       </c>
     </row>
@@ -3882,11 +3882,11 @@
         </is>
       </c>
       <c r="H7" s="7">
-        <f>SUMIFS($D$5:$D$1000,$C$5:$C$1000,G7,$A$5:$A$1000,_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G7))</f>
+        <f>IF(I7=0,"",SUMIFS($D$5:$D$1000,$C$5:$C$1000,G7,$A$5:$A$1000,I7))</f>
         <v/>
       </c>
       <c r="I7" s="11">
-        <f>_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G7)</f>
+        <f>SUMPRODUCT(MAX(($C$5:$C$1000=G7)*$A$5:$A$1000))</f>
         <v/>
       </c>
     </row>
@@ -3918,11 +3918,11 @@
         </is>
       </c>
       <c r="H8" s="7">
-        <f>SUMIFS($D$5:$D$1000,$C$5:$C$1000,G8,$A$5:$A$1000,_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G8))</f>
+        <f>IF(I8=0,"",SUMIFS($D$5:$D$1000,$C$5:$C$1000,G8,$A$5:$A$1000,I8))</f>
         <v/>
       </c>
       <c r="I8" s="11">
-        <f>_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G8)</f>
+        <f>SUMPRODUCT(MAX(($C$5:$C$1000=G8)*$A$5:$A$1000))</f>
         <v/>
       </c>
     </row>
@@ -3954,11 +3954,11 @@
         </is>
       </c>
       <c r="H9" s="7">
-        <f>SUMIFS($D$5:$D$1000,$C$5:$C$1000,G9,$A$5:$A$1000,_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G9))</f>
+        <f>IF(I9=0,"",SUMIFS($D$5:$D$1000,$C$5:$C$1000,G9,$A$5:$A$1000,I9))</f>
         <v/>
       </c>
       <c r="I9" s="11">
-        <f>_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G9)</f>
+        <f>SUMPRODUCT(MAX(($C$5:$C$1000=G9)*$A$5:$A$1000))</f>
         <v/>
       </c>
     </row>
@@ -3990,11 +3990,11 @@
         </is>
       </c>
       <c r="H10" s="7">
-        <f>SUMIFS($D$5:$D$1000,$C$5:$C$1000,G10,$A$5:$A$1000,_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G10))</f>
+        <f>IF(I10=0,"",SUMIFS($D$5:$D$1000,$C$5:$C$1000,G10,$A$5:$A$1000,I10))</f>
         <v/>
       </c>
       <c r="I10" s="11">
-        <f>_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G10)</f>
+        <f>SUMPRODUCT(MAX(($C$5:$C$1000=G10)*$A$5:$A$1000))</f>
         <v/>
       </c>
     </row>
@@ -4026,11 +4026,11 @@
         </is>
       </c>
       <c r="H11" s="7">
-        <f>SUMIFS($D$5:$D$1000,$C$5:$C$1000,G11,$A$5:$A$1000,_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G11))</f>
+        <f>IF(I11=0,"",SUMIFS($D$5:$D$1000,$C$5:$C$1000,G11,$A$5:$A$1000,I11))</f>
         <v/>
       </c>
       <c r="I11" s="11">
-        <f>_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G11)</f>
+        <f>SUMPRODUCT(MAX(($C$5:$C$1000=G11)*$A$5:$A$1000))</f>
         <v/>
       </c>
     </row>
@@ -4062,11 +4062,11 @@
         </is>
       </c>
       <c r="H12" s="7">
-        <f>SUMIFS($D$5:$D$1000,$C$5:$C$1000,G12,$A$5:$A$1000,_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G12))</f>
+        <f>IF(I12=0,"",SUMIFS($D$5:$D$1000,$C$5:$C$1000,G12,$A$5:$A$1000,I12))</f>
         <v/>
       </c>
       <c r="I12" s="11">
-        <f>_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G12)</f>
+        <f>SUMPRODUCT(MAX(($C$5:$C$1000=G12)*$A$5:$A$1000))</f>
         <v/>
       </c>
     </row>
@@ -4098,11 +4098,11 @@
         </is>
       </c>
       <c r="H13" s="7">
-        <f>SUMIFS($D$5:$D$1000,$C$5:$C$1000,G13,$A$5:$A$1000,_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G13))</f>
+        <f>IF(I13=0,"",SUMIFS($D$5:$D$1000,$C$5:$C$1000,G13,$A$5:$A$1000,I13))</f>
         <v/>
       </c>
       <c r="I13" s="11">
-        <f>_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G13)</f>
+        <f>SUMPRODUCT(MAX(($C$5:$C$1000=G13)*$A$5:$A$1000))</f>
         <v/>
       </c>
     </row>
@@ -4134,11 +4134,11 @@
         </is>
       </c>
       <c r="H14" s="7">
-        <f>SUMIFS($D$5:$D$1000,$C$5:$C$1000,G14,$A$5:$A$1000,_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G14))</f>
+        <f>IF(I14=0,"",SUMIFS($D$5:$D$1000,$C$5:$C$1000,G14,$A$5:$A$1000,I14))</f>
         <v/>
       </c>
       <c r="I14" s="11">
-        <f>_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G14)</f>
+        <f>SUMPRODUCT(MAX(($C$5:$C$1000=G14)*$A$5:$A$1000))</f>
         <v/>
       </c>
     </row>
@@ -4170,11 +4170,11 @@
         </is>
       </c>
       <c r="H15" s="7">
-        <f>SUMIFS($D$5:$D$1000,$C$5:$C$1000,G15,$A$5:$A$1000,_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G15))</f>
+        <f>IF(I15=0,"",SUMIFS($D$5:$D$1000,$C$5:$C$1000,G15,$A$5:$A$1000,I15))</f>
         <v/>
       </c>
       <c r="I15" s="11">
-        <f>_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G15)</f>
+        <f>SUMPRODUCT(MAX(($C$5:$C$1000=G15)*$A$5:$A$1000))</f>
         <v/>
       </c>
     </row>
@@ -4202,11 +4202,11 @@
         </is>
       </c>
       <c r="H16" s="7">
-        <f>SUMIFS($D$5:$D$1000,$C$5:$C$1000,G16,$A$5:$A$1000,_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G16))</f>
+        <f>IF(I16=0,"",SUMIFS($D$5:$D$1000,$C$5:$C$1000,G16,$A$5:$A$1000,I16))</f>
         <v/>
       </c>
       <c r="I16" s="11">
-        <f>_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G16)</f>
+        <f>SUMPRODUCT(MAX(($C$5:$C$1000=G16)*$A$5:$A$1000))</f>
         <v/>
       </c>
     </row>
@@ -4234,11 +4234,11 @@
         </is>
       </c>
       <c r="H17" s="7">
-        <f>SUMIFS($D$5:$D$1000,$C$5:$C$1000,G17,$A$5:$A$1000,_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G17))</f>
+        <f>IF(I17=0,"",SUMIFS($D$5:$D$1000,$C$5:$C$1000,G17,$A$5:$A$1000,I17))</f>
         <v/>
       </c>
       <c r="I17" s="11">
-        <f>_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G17)</f>
+        <f>SUMPRODUCT(MAX(($C$5:$C$1000=G17)*$A$5:$A$1000))</f>
         <v/>
       </c>
     </row>
@@ -4266,11 +4266,11 @@
         </is>
       </c>
       <c r="H18" s="7">
-        <f>SUMIFS($D$5:$D$1000,$C$5:$C$1000,G18,$A$5:$A$1000,_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G18))</f>
+        <f>IF(I18=0,"",SUMIFS($D$5:$D$1000,$C$5:$C$1000,G18,$A$5:$A$1000,I18))</f>
         <v/>
       </c>
       <c r="I18" s="11">
-        <f>_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G18)</f>
+        <f>SUMPRODUCT(MAX(($C$5:$C$1000=G18)*$A$5:$A$1000))</f>
         <v/>
       </c>
     </row>
@@ -4302,11 +4302,11 @@
         </is>
       </c>
       <c r="H19" s="7">
-        <f>SUMIFS($D$5:$D$1000,$C$5:$C$1000,G19,$A$5:$A$1000,_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G19))</f>
+        <f>IF(I19=0,"",SUMIFS($D$5:$D$1000,$C$5:$C$1000,G19,$A$5:$A$1000,I19))</f>
         <v/>
       </c>
       <c r="I19" s="11">
-        <f>_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G19)</f>
+        <f>SUMPRODUCT(MAX(($C$5:$C$1000=G19)*$A$5:$A$1000))</f>
         <v/>
       </c>
     </row>
@@ -4338,11 +4338,11 @@
         </is>
       </c>
       <c r="H20" s="7">
-        <f>SUMIFS($D$5:$D$1000,$C$5:$C$1000,G20,$A$5:$A$1000,_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G20))</f>
+        <f>IF(I20=0,"",SUMIFS($D$5:$D$1000,$C$5:$C$1000,G20,$A$5:$A$1000,I20))</f>
         <v/>
       </c>
       <c r="I20" s="11">
-        <f>_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G20)</f>
+        <f>SUMPRODUCT(MAX(($C$5:$C$1000=G20)*$A$5:$A$1000))</f>
         <v/>
       </c>
     </row>
@@ -4374,11 +4374,11 @@
         </is>
       </c>
       <c r="H21" s="7">
-        <f>SUMIFS($D$5:$D$1000,$C$5:$C$1000,G21,$A$5:$A$1000,_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G21))</f>
+        <f>IF(I21=0,"",SUMIFS($D$5:$D$1000,$C$5:$C$1000,G21,$A$5:$A$1000,I21))</f>
         <v/>
       </c>
       <c r="I21" s="11">
-        <f>_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G21)</f>
+        <f>SUMPRODUCT(MAX(($C$5:$C$1000=G21)*$A$5:$A$1000))</f>
         <v/>
       </c>
     </row>
@@ -4410,11 +4410,11 @@
         </is>
       </c>
       <c r="H22" s="7">
-        <f>SUMIFS($D$5:$D$1000,$C$5:$C$1000,G22,$A$5:$A$1000,_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G22))</f>
+        <f>IF(I22=0,"",SUMIFS($D$5:$D$1000,$C$5:$C$1000,G22,$A$5:$A$1000,I22))</f>
         <v/>
       </c>
       <c r="I22" s="11">
-        <f>_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G22)</f>
+        <f>SUMPRODUCT(MAX(($C$5:$C$1000=G22)*$A$5:$A$1000))</f>
         <v/>
       </c>
     </row>
@@ -4446,11 +4446,11 @@
         </is>
       </c>
       <c r="H23" s="7">
-        <f>SUMIFS($D$5:$D$1000,$C$5:$C$1000,G23,$A$5:$A$1000,_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G23))</f>
+        <f>IF(I23=0,"",SUMIFS($D$5:$D$1000,$C$5:$C$1000,G23,$A$5:$A$1000,I23))</f>
         <v/>
       </c>
       <c r="I23" s="11">
-        <f>_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G23)</f>
+        <f>SUMPRODUCT(MAX(($C$5:$C$1000=G23)*$A$5:$A$1000))</f>
         <v/>
       </c>
     </row>
@@ -4478,11 +4478,11 @@
         </is>
       </c>
       <c r="H24" s="7">
-        <f>SUMIFS($D$5:$D$1000,$C$5:$C$1000,G24,$A$5:$A$1000,_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G24))</f>
+        <f>IF(I24=0,"",SUMIFS($D$5:$D$1000,$C$5:$C$1000,G24,$A$5:$A$1000,I24))</f>
         <v/>
       </c>
       <c r="I24" s="11">
-        <f>_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G24)</f>
+        <f>SUMPRODUCT(MAX(($C$5:$C$1000=G24)*$A$5:$A$1000))</f>
         <v/>
       </c>
     </row>
@@ -4514,11 +4514,11 @@
         </is>
       </c>
       <c r="H25" s="7">
-        <f>SUMIFS($D$5:$D$1000,$C$5:$C$1000,G25,$A$5:$A$1000,_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G25))</f>
+        <f>IF(I25=0,"",SUMIFS($D$5:$D$1000,$C$5:$C$1000,G25,$A$5:$A$1000,I25))</f>
         <v/>
       </c>
       <c r="I25" s="11">
-        <f>_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G25)</f>
+        <f>SUMPRODUCT(MAX(($C$5:$C$1000=G25)*$A$5:$A$1000))</f>
         <v/>
       </c>
     </row>
@@ -4546,11 +4546,11 @@
         </is>
       </c>
       <c r="H26" s="7">
-        <f>SUMIFS($D$5:$D$1000,$C$5:$C$1000,G26,$A$5:$A$1000,_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G26))</f>
+        <f>IF(I26=0,"",SUMIFS($D$5:$D$1000,$C$5:$C$1000,G26,$A$5:$A$1000,I26))</f>
         <v/>
       </c>
       <c r="I26" s="11">
-        <f>_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G26)</f>
+        <f>SUMPRODUCT(MAX(($C$5:$C$1000=G26)*$A$5:$A$1000))</f>
         <v/>
       </c>
     </row>
@@ -4582,11 +4582,11 @@
         </is>
       </c>
       <c r="H27" s="7">
-        <f>SUMIFS($D$5:$D$1000,$C$5:$C$1000,G27,$A$5:$A$1000,_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G27))</f>
+        <f>IF(I27=0,"",SUMIFS($D$5:$D$1000,$C$5:$C$1000,G27,$A$5:$A$1000,I27))</f>
         <v/>
       </c>
       <c r="I27" s="11">
-        <f>_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G27)</f>
+        <f>SUMPRODUCT(MAX(($C$5:$C$1000=G27)*$A$5:$A$1000))</f>
         <v/>
       </c>
     </row>
@@ -4618,11 +4618,11 @@
         </is>
       </c>
       <c r="H28" s="7">
-        <f>SUMIFS($D$5:$D$1000,$C$5:$C$1000,G28,$A$5:$A$1000,_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G28))</f>
+        <f>IF(I28=0,"",SUMIFS($D$5:$D$1000,$C$5:$C$1000,G28,$A$5:$A$1000,I28))</f>
         <v/>
       </c>
       <c r="I28" s="11">
-        <f>_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G28)</f>
+        <f>SUMPRODUCT(MAX(($C$5:$C$1000=G28)*$A$5:$A$1000))</f>
         <v/>
       </c>
     </row>
@@ -4650,11 +4650,11 @@
         </is>
       </c>
       <c r="H29" s="7">
-        <f>SUMIFS($D$5:$D$1000,$C$5:$C$1000,G29,$A$5:$A$1000,_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G29))</f>
+        <f>IF(I29=0,"",SUMIFS($D$5:$D$1000,$C$5:$C$1000,G29,$A$5:$A$1000,I29))</f>
         <v/>
       </c>
       <c r="I29" s="11">
-        <f>_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G29)</f>
+        <f>SUMPRODUCT(MAX(($C$5:$C$1000=G29)*$A$5:$A$1000))</f>
         <v/>
       </c>
     </row>
@@ -4686,11 +4686,11 @@
         </is>
       </c>
       <c r="H30" s="7">
-        <f>SUMIFS($D$5:$D$1000,$C$5:$C$1000,G30,$A$5:$A$1000,_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G30))</f>
+        <f>IF(I30=0,"",SUMIFS($D$5:$D$1000,$C$5:$C$1000,G30,$A$5:$A$1000,I30))</f>
         <v/>
       </c>
       <c r="I30" s="11">
-        <f>_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G30)</f>
+        <f>SUMPRODUCT(MAX(($C$5:$C$1000=G30)*$A$5:$A$1000))</f>
         <v/>
       </c>
     </row>
@@ -4722,11 +4722,11 @@
         </is>
       </c>
       <c r="H31" s="7">
-        <f>SUMIFS($D$5:$D$1000,$C$5:$C$1000,G31,$A$5:$A$1000,_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G31))</f>
+        <f>IF(I31=0,"",SUMIFS($D$5:$D$1000,$C$5:$C$1000,G31,$A$5:$A$1000,I31))</f>
         <v/>
       </c>
       <c r="I31" s="11">
-        <f>_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G31)</f>
+        <f>SUMPRODUCT(MAX(($C$5:$C$1000=G31)*$A$5:$A$1000))</f>
         <v/>
       </c>
     </row>
@@ -4758,11 +4758,11 @@
         </is>
       </c>
       <c r="H32" s="7">
-        <f>SUMIFS($D$5:$D$1000,$C$5:$C$1000,G32,$A$5:$A$1000,_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G32))</f>
+        <f>IF(I32=0,"",SUMIFS($D$5:$D$1000,$C$5:$C$1000,G32,$A$5:$A$1000,I32))</f>
         <v/>
       </c>
       <c r="I32" s="11">
-        <f>_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G32)</f>
+        <f>SUMPRODUCT(MAX(($C$5:$C$1000=G32)*$A$5:$A$1000))</f>
         <v/>
       </c>
     </row>
@@ -4794,11 +4794,11 @@
         </is>
       </c>
       <c r="H33" s="7">
-        <f>SUMIFS($D$5:$D$1000,$C$5:$C$1000,G33,$A$5:$A$1000,_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G33))</f>
+        <f>IF(I33=0,"",SUMIFS($D$5:$D$1000,$C$5:$C$1000,G33,$A$5:$A$1000,I33))</f>
         <v/>
       </c>
       <c r="I33" s="11">
-        <f>_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G33)</f>
+        <f>SUMPRODUCT(MAX(($C$5:$C$1000=G33)*$A$5:$A$1000))</f>
         <v/>
       </c>
     </row>
@@ -4830,14 +4830,15 @@
         </is>
       </c>
       <c r="H34" s="7">
-        <f>SUMIFS($D$5:$D$1000,$C$5:$C$1000,G34,$A$5:$A$1000,_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G34))</f>
+        <f>IF(I34=0,"",SUMIFS($D$5:$D$1000,$C$5:$C$1000,G34,$A$5:$A$1000,I34))</f>
         <v/>
       </c>
       <c r="I34" s="11">
-        <f>_xlfn.MAXIFS($A$5:$A$1000,$C$5:$C$1000,G34)</f>
-        <v/>
-      </c>
-    </row>
+        <f>SUMPRODUCT(MAX(($C$5:$C$1000=G34)*$A$5:$A$1000))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35"/>
     <row r="36">
       <c r="A36" s="12" t="inlineStr">
         <is>
@@ -4845,6 +4846,169 @@
         </is>
       </c>
     </row>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
+    <row r="88"/>
+    <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94"/>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97"/>
+    <row r="98"/>
+    <row r="99"/>
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102"/>
+    <row r="103"/>
+    <row r="104"/>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
+    <row r="108"/>
+    <row r="109"/>
+    <row r="110"/>
+    <row r="111"/>
+    <row r="112"/>
+    <row r="113"/>
+    <row r="114"/>
+    <row r="115"/>
+    <row r="116"/>
+    <row r="117"/>
+    <row r="118"/>
+    <row r="119"/>
+    <row r="120"/>
+    <row r="121"/>
+    <row r="122"/>
+    <row r="123"/>
+    <row r="124"/>
+    <row r="125"/>
+    <row r="126"/>
+    <row r="127"/>
+    <row r="128"/>
+    <row r="129"/>
+    <row r="130"/>
+    <row r="131"/>
+    <row r="132"/>
+    <row r="133"/>
+    <row r="134"/>
+    <row r="135"/>
+    <row r="136"/>
+    <row r="137"/>
+    <row r="138"/>
+    <row r="139"/>
+    <row r="140"/>
+    <row r="141"/>
+    <row r="142"/>
+    <row r="143"/>
+    <row r="144"/>
+    <row r="145"/>
+    <row r="146"/>
+    <row r="147"/>
+    <row r="148"/>
+    <row r="149"/>
+    <row r="150"/>
+    <row r="151"/>
+    <row r="152"/>
+    <row r="153"/>
+    <row r="154"/>
+    <row r="155"/>
+    <row r="156"/>
+    <row r="157"/>
+    <row r="158"/>
+    <row r="159"/>
+    <row r="160"/>
+    <row r="161"/>
+    <row r="162"/>
+    <row r="163"/>
+    <row r="164"/>
+    <row r="165"/>
+    <row r="166"/>
+    <row r="167"/>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183"/>
+    <row r="184"/>
+    <row r="185"/>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:L2"/>

</xml_diff>

<commit_message>
Correct the AI Mode tally: six of six, not five
The manual re-run of the freelancer-cost query showed Google AI Mode naming
Design Bees and citing the site more than any other source. Appendix J1
already recorded 6/6 for AI Mode and 5/6 for ChatGPT; the one-line read at
the top still said "each ... five of six". Fixed, and the Tracking tab's
11 Sep AI Mode reading goes from 5 to 6.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MUHUj2RPRZAnBNADpTZfsW
</commit_message>
<xml_diff>
--- a/docs/seo/designbees-aeo-seo-tracker-2026-09-10.xlsx
+++ b/docs/seo/designbees-aeo-seo-tracker-2026-09-10.xlsx
@@ -5051,11 +5051,11 @@
         </is>
       </c>
       <c r="D37" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>11 Sep live check</t>
+          <t>11 Sep live check; includes the freelancer query, won on AI Mode</t>
         </is>
       </c>
     </row>

</xml_diff>